<commit_message>
feat: update fetch-worker.js configuration and add sync-results.js for Excel output
</commit_message>
<xml_diff>
--- a/volume/output_manual.xlsx
+++ b/volume/output_manual.xlsx
@@ -3151,6 +3151,9 @@
       <c r="P52" t="str">
         <v>Add</v>
       </c>
+      <c r="Q52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3201,6 +3204,9 @@
       <c r="P53" t="str">
         <v>Add</v>
       </c>
+      <c r="Q53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3251,6 +3257,9 @@
       <c r="P54" t="str">
         <v>Add</v>
       </c>
+      <c r="Q54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3301,6 +3310,9 @@
       <c r="P55" t="str">
         <v>Add</v>
       </c>
+      <c r="Q55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3351,6 +3363,9 @@
       <c r="P56" t="str">
         <v>Add</v>
       </c>
+      <c r="Q56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3401,6 +3416,9 @@
       <c r="P57" t="str">
         <v>Add</v>
       </c>
+      <c r="Q57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3451,6 +3469,9 @@
       <c r="P58" t="str">
         <v>Add</v>
       </c>
+      <c r="Q58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3501,6 +3522,9 @@
       <c r="P59" t="str">
         <v>Add</v>
       </c>
+      <c r="Q59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3551,6 +3575,9 @@
       <c r="P60" t="str">
         <v>Add</v>
       </c>
+      <c r="Q60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3601,6 +3628,9 @@
       <c r="P61" t="str">
         <v>Add</v>
       </c>
+      <c r="Q61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3651,6 +3681,9 @@
       <c r="P62" t="str">
         <v>Add</v>
       </c>
+      <c r="Q62" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3701,6 +3734,9 @@
       <c r="P63" t="str">
         <v>Add</v>
       </c>
+      <c r="Q63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3751,6 +3787,9 @@
       <c r="P64" t="str">
         <v>Add</v>
       </c>
+      <c r="Q64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3801,6 +3840,9 @@
       <c r="P65" t="str">
         <v>Add</v>
       </c>
+      <c r="Q65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3851,6 +3893,9 @@
       <c r="P66" t="str">
         <v>Add</v>
       </c>
+      <c r="Q66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3901,6 +3946,9 @@
       <c r="P67" t="str">
         <v>Add</v>
       </c>
+      <c r="Q67" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3951,6 +3999,9 @@
       <c r="P68" t="str">
         <v>Add</v>
       </c>
+      <c r="Q68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -4001,6 +4052,9 @@
       <c r="P69" t="str">
         <v>Add</v>
       </c>
+      <c r="Q69" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -4051,6 +4105,9 @@
       <c r="P70" t="str">
         <v>Add</v>
       </c>
+      <c r="Q70" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -4101,6 +4158,9 @@
       <c r="P71" t="str">
         <v>Add</v>
       </c>
+      <c r="Q71" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -4151,6 +4211,9 @@
       <c r="P72" t="str">
         <v>Add</v>
       </c>
+      <c r="Q72" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4201,6 +4264,9 @@
       <c r="P73" t="str">
         <v>Add</v>
       </c>
+      <c r="Q73" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4251,6 +4317,9 @@
       <c r="P74" t="str">
         <v>Add</v>
       </c>
+      <c r="Q74" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4301,6 +4370,9 @@
       <c r="P75" t="str">
         <v>Add</v>
       </c>
+      <c r="Q75" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4351,6 +4423,9 @@
       <c r="P76" t="str">
         <v>Add</v>
       </c>
+      <c r="Q76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4401,6 +4476,9 @@
       <c r="P77" t="str">
         <v>Add</v>
       </c>
+      <c r="Q77" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4451,6 +4529,9 @@
       <c r="P78" t="str">
         <v>Add</v>
       </c>
+      <c r="Q78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -4501,6 +4582,9 @@
       <c r="P79" t="str">
         <v>Add</v>
       </c>
+      <c r="Q79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4551,6 +4635,9 @@
       <c r="P80" t="str">
         <v>Add</v>
       </c>
+      <c r="Q80" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -4601,6 +4688,9 @@
       <c r="P81" t="str">
         <v>Add</v>
       </c>
+      <c r="Q81" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4651,6 +4741,9 @@
       <c r="P82" t="str">
         <v>Add</v>
       </c>
+      <c r="Q82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4701,6 +4794,9 @@
       <c r="P83" t="str">
         <v>Add</v>
       </c>
+      <c r="Q83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4751,6 +4847,9 @@
       <c r="P84" t="str">
         <v>Add</v>
       </c>
+      <c r="Q84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4801,6 +4900,9 @@
       <c r="P85" t="str">
         <v>Add</v>
       </c>
+      <c r="Q85" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4851,6 +4953,9 @@
       <c r="P86" t="str">
         <v>Add</v>
       </c>
+      <c r="Q86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4901,6 +5006,9 @@
       <c r="P87" t="str">
         <v>Add</v>
       </c>
+      <c r="Q87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4951,6 +5059,9 @@
       <c r="P88" t="str">
         <v>Add</v>
       </c>
+      <c r="Q88" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -5001,6 +5112,9 @@
       <c r="P89" t="str">
         <v>Add</v>
       </c>
+      <c r="Q89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5051,6 +5165,9 @@
       <c r="P90" t="str">
         <v>Add</v>
       </c>
+      <c r="Q90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5101,6 +5218,9 @@
       <c r="P91" t="str">
         <v>Add</v>
       </c>
+      <c r="Q91" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -5151,6 +5271,9 @@
       <c r="P92" t="str">
         <v>Add</v>
       </c>
+      <c r="Q92" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5201,6 +5324,9 @@
       <c r="P93" t="str">
         <v>Add</v>
       </c>
+      <c r="Q93" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5251,6 +5377,9 @@
       <c r="P94" t="str">
         <v>Add</v>
       </c>
+      <c r="Q94" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5301,6 +5430,9 @@
       <c r="P95" t="str">
         <v>Add</v>
       </c>
+      <c r="Q95" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5351,6 +5483,9 @@
       <c r="P96" t="str">
         <v>Add</v>
       </c>
+      <c r="Q96" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5401,6 +5536,9 @@
       <c r="P97" t="str">
         <v>Add</v>
       </c>
+      <c r="Q97" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5451,6 +5589,9 @@
       <c r="P98" t="str">
         <v>Add</v>
       </c>
+      <c r="Q98" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5501,6 +5642,9 @@
       <c r="P99" t="str">
         <v>Add</v>
       </c>
+      <c r="Q99" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -5551,6 +5695,9 @@
       <c r="P100" t="str">
         <v>Add</v>
       </c>
+      <c r="Q100" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5600,6 +5747,9 @@
       </c>
       <c r="P101" t="str">
         <v>Add</v>
+      </c>
+      <c r="Q101" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="102">

</xml_diff>

<commit_message>
feat: update bearer token in fetch-worker.js and add new results to JSON output
</commit_message>
<xml_diff>
--- a/volume/output_manual.xlsx
+++ b/volume/output_manual.xlsx
@@ -5801,6 +5801,9 @@
       <c r="P102" t="str">
         <v>Add</v>
       </c>
+      <c r="Q102" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -5851,6 +5854,9 @@
       <c r="P103" t="str">
         <v>Add</v>
       </c>
+      <c r="Q103" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -5901,6 +5907,9 @@
       <c r="P104" t="str">
         <v>Add</v>
       </c>
+      <c r="Q104" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -5951,6 +5960,9 @@
       <c r="P105" t="str">
         <v>Add</v>
       </c>
+      <c r="Q105" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -6001,6 +6013,9 @@
       <c r="P106" t="str">
         <v>Add</v>
       </c>
+      <c r="Q106" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -6051,6 +6066,9 @@
       <c r="P107" t="str">
         <v>Add</v>
       </c>
+      <c r="Q107" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -6101,6 +6119,9 @@
       <c r="P108" t="str">
         <v>Add</v>
       </c>
+      <c r="Q108" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -6151,6 +6172,9 @@
       <c r="P109" t="str">
         <v>Add</v>
       </c>
+      <c r="Q109" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -6201,6 +6225,9 @@
       <c r="P110" t="str">
         <v>Add</v>
       </c>
+      <c r="Q110" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -6251,6 +6278,9 @@
       <c r="P111" t="str">
         <v>Add</v>
       </c>
+      <c r="Q111" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -6301,6 +6331,9 @@
       <c r="P112" t="str">
         <v>Add</v>
       </c>
+      <c r="Q112" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -6351,6 +6384,9 @@
       <c r="P113" t="str">
         <v>Add</v>
       </c>
+      <c r="Q113" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -6401,6 +6437,9 @@
       <c r="P114" t="str">
         <v>Add</v>
       </c>
+      <c r="Q114" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -6451,6 +6490,9 @@
       <c r="P115" t="str">
         <v>Add</v>
       </c>
+      <c r="Q115" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -6501,6 +6543,9 @@
       <c r="P116" t="str">
         <v>Add</v>
       </c>
+      <c r="Q116" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -6551,6 +6596,9 @@
       <c r="P117" t="str">
         <v>Add</v>
       </c>
+      <c r="Q117" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -6601,6 +6649,9 @@
       <c r="P118" t="str">
         <v>Add</v>
       </c>
+      <c r="Q118" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -6651,6 +6702,9 @@
       <c r="P119" t="str">
         <v>Add</v>
       </c>
+      <c r="Q119" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -6701,6 +6755,9 @@
       <c r="P120" t="str">
         <v>Add</v>
       </c>
+      <c r="Q120" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -6751,6 +6808,9 @@
       <c r="P121" t="str">
         <v>Add</v>
       </c>
+      <c r="Q121" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -6801,6 +6861,9 @@
       <c r="P122" t="str">
         <v>Add</v>
       </c>
+      <c r="Q122" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -6851,6 +6914,9 @@
       <c r="P123" t="str">
         <v>Add</v>
       </c>
+      <c r="Q123" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -6901,6 +6967,9 @@
       <c r="P124" t="str">
         <v>Add</v>
       </c>
+      <c r="Q124" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -6951,6 +7020,9 @@
       <c r="P125" t="str">
         <v>Add</v>
       </c>
+      <c r="Q125" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -7001,6 +7073,9 @@
       <c r="P126" t="str">
         <v>Add</v>
       </c>
+      <c r="Q126" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -7051,6 +7126,9 @@
       <c r="P127" t="str">
         <v>Add</v>
       </c>
+      <c r="Q127" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -7101,6 +7179,9 @@
       <c r="P128" t="str">
         <v>Add</v>
       </c>
+      <c r="Q128" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -7151,6 +7232,9 @@
       <c r="P129" t="str">
         <v>Add</v>
       </c>
+      <c r="Q129" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -7201,6 +7285,9 @@
       <c r="P130" t="str">
         <v>Add</v>
       </c>
+      <c r="Q130" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -7251,6 +7338,9 @@
       <c r="P131" t="str">
         <v>Add</v>
       </c>
+      <c r="Q131" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -7301,6 +7391,9 @@
       <c r="P132" t="str">
         <v>Add</v>
       </c>
+      <c r="Q132" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -7351,6 +7444,9 @@
       <c r="P133" t="str">
         <v>Add</v>
       </c>
+      <c r="Q133" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -7401,6 +7497,9 @@
       <c r="P134" t="str">
         <v>Add</v>
       </c>
+      <c r="Q134" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -7451,6 +7550,9 @@
       <c r="P135" t="str">
         <v>Add</v>
       </c>
+      <c r="Q135" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -7501,6 +7603,9 @@
       <c r="P136" t="str">
         <v>Add</v>
       </c>
+      <c r="Q136" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -7551,6 +7656,9 @@
       <c r="P137" t="str">
         <v>Add</v>
       </c>
+      <c r="Q137" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -7601,6 +7709,9 @@
       <c r="P138" t="str">
         <v>Add</v>
       </c>
+      <c r="Q138" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -7651,6 +7762,9 @@
       <c r="P139" t="str">
         <v>Add</v>
       </c>
+      <c r="Q139" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -7701,6 +7815,9 @@
       <c r="P140" t="str">
         <v>Add</v>
       </c>
+      <c r="Q140" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -7751,6 +7868,9 @@
       <c r="P141" t="str">
         <v>Add</v>
       </c>
+      <c r="Q141" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -7801,6 +7921,9 @@
       <c r="P142" t="str">
         <v>Add</v>
       </c>
+      <c r="Q142" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -7851,6 +7974,9 @@
       <c r="P143" t="str">
         <v>Add</v>
       </c>
+      <c r="Q143" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -7901,6 +8027,9 @@
       <c r="P144" t="str">
         <v>Add</v>
       </c>
+      <c r="Q144" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -7951,6 +8080,9 @@
       <c r="P145" t="str">
         <v>Add</v>
       </c>
+      <c r="Q145" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -8001,6 +8133,9 @@
       <c r="P146" t="str">
         <v>Add</v>
       </c>
+      <c r="Q146" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -8051,6 +8186,9 @@
       <c r="P147" t="str">
         <v>Add</v>
       </c>
+      <c r="Q147" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -8101,6 +8239,9 @@
       <c r="P148" t="str">
         <v>Add</v>
       </c>
+      <c r="Q148" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -8151,6 +8292,9 @@
       <c r="P149" t="str">
         <v>Add</v>
       </c>
+      <c r="Q149" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -8200,6 +8344,9 @@
       </c>
       <c r="P150" t="str">
         <v>Add</v>
+      </c>
+      <c r="Q150" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="151">

</xml_diff>

<commit_message>
feat: update row range in fetch-worker.js and add new results to results_manual.json
</commit_message>
<xml_diff>
--- a/volume/output_manual.xlsx
+++ b/volume/output_manual.xlsx
@@ -8448,6 +8448,9 @@
       <c r="P152" t="str">
         <v>Add</v>
       </c>
+      <c r="Q152" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -8498,6 +8501,9 @@
       <c r="P153" t="str">
         <v>Add</v>
       </c>
+      <c r="Q153" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -8548,6 +8554,9 @@
       <c r="P154" t="str">
         <v>Add</v>
       </c>
+      <c r="Q154" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -8598,6 +8607,9 @@
       <c r="P155" t="str">
         <v>Add</v>
       </c>
+      <c r="Q155" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -8648,6 +8660,9 @@
       <c r="P156" t="str">
         <v>Add</v>
       </c>
+      <c r="Q156" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -8698,6 +8713,9 @@
       <c r="P157" t="str">
         <v>Add</v>
       </c>
+      <c r="Q157" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -8748,6 +8766,9 @@
       <c r="P158" t="str">
         <v>Add</v>
       </c>
+      <c r="Q158" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -8798,6 +8819,9 @@
       <c r="P159" t="str">
         <v>Add</v>
       </c>
+      <c r="Q159" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -8848,6 +8872,9 @@
       <c r="P160" t="str">
         <v>Add</v>
       </c>
+      <c r="Q160" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -8898,6 +8925,9 @@
       <c r="P161" t="str">
         <v>Add</v>
       </c>
+      <c r="Q161" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -8948,6 +8978,9 @@
       <c r="P162" t="str">
         <v>Add</v>
       </c>
+      <c r="Q162" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -8998,6 +9031,9 @@
       <c r="P163" t="str">
         <v>Add</v>
       </c>
+      <c r="Q163" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -9048,6 +9084,9 @@
       <c r="P164" t="str">
         <v>Add</v>
       </c>
+      <c r="Q164" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -9098,6 +9137,9 @@
       <c r="P165" t="str">
         <v>Add</v>
       </c>
+      <c r="Q165" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -9148,6 +9190,9 @@
       <c r="P166" t="str">
         <v>Add</v>
       </c>
+      <c r="Q166" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -9198,6 +9243,9 @@
       <c r="P167" t="str">
         <v>Add</v>
       </c>
+      <c r="Q167" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -9248,6 +9296,9 @@
       <c r="P168" t="str">
         <v>Add</v>
       </c>
+      <c r="Q168" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -9298,6 +9349,9 @@
       <c r="P169" t="str">
         <v>Add</v>
       </c>
+      <c r="Q169" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -9348,6 +9402,9 @@
       <c r="P170" t="str">
         <v>Add</v>
       </c>
+      <c r="Q170" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -9398,6 +9455,9 @@
       <c r="P171" t="str">
         <v>Add</v>
       </c>
+      <c r="Q171" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -9448,6 +9508,9 @@
       <c r="P172" t="str">
         <v>Add</v>
       </c>
+      <c r="Q172" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -9498,6 +9561,9 @@
       <c r="P173" t="str">
         <v>Add</v>
       </c>
+      <c r="Q173" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -9548,6 +9614,9 @@
       <c r="P174" t="str">
         <v>Add</v>
       </c>
+      <c r="Q174" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -9598,6 +9667,9 @@
       <c r="P175" t="str">
         <v>Add</v>
       </c>
+      <c r="Q175" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -9648,6 +9720,9 @@
       <c r="P176" t="str">
         <v>Add</v>
       </c>
+      <c r="Q176" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -9698,6 +9773,9 @@
       <c r="P177" t="str">
         <v>Add</v>
       </c>
+      <c r="Q177" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -9748,6 +9826,9 @@
       <c r="P178" t="str">
         <v>Add</v>
       </c>
+      <c r="Q178" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -9798,6 +9879,9 @@
       <c r="P179" t="str">
         <v>Add</v>
       </c>
+      <c r="Q179" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -9848,6 +9932,9 @@
       <c r="P180" t="str">
         <v>Add</v>
       </c>
+      <c r="Q180" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -9898,6 +9985,9 @@
       <c r="P181" t="str">
         <v>Add</v>
       </c>
+      <c r="Q181" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -9948,6 +10038,9 @@
       <c r="P182" t="str">
         <v>Add</v>
       </c>
+      <c r="Q182" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -9998,6 +10091,9 @@
       <c r="P183" t="str">
         <v>Add</v>
       </c>
+      <c r="Q183" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -10048,6 +10144,9 @@
       <c r="P184" t="str">
         <v>Add</v>
       </c>
+      <c r="Q184" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -10098,6 +10197,9 @@
       <c r="P185" t="str">
         <v>Add</v>
       </c>
+      <c r="Q185" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -10148,6 +10250,9 @@
       <c r="P186" t="str">
         <v>Add</v>
       </c>
+      <c r="Q186" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -10198,6 +10303,9 @@
       <c r="P187" t="str">
         <v>Add</v>
       </c>
+      <c r="Q187" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -10248,6 +10356,9 @@
       <c r="P188" t="str">
         <v>Add</v>
       </c>
+      <c r="Q188" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -10298,6 +10409,9 @@
       <c r="P189" t="str">
         <v>Add</v>
       </c>
+      <c r="Q189" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -10348,6 +10462,9 @@
       <c r="P190" t="str">
         <v>Add</v>
       </c>
+      <c r="Q190" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -10398,6 +10515,9 @@
       <c r="P191" t="str">
         <v>Add</v>
       </c>
+      <c r="Q191" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -10448,6 +10568,9 @@
       <c r="P192" t="str">
         <v>Add</v>
       </c>
+      <c r="Q192" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -10498,6 +10621,9 @@
       <c r="P193" t="str">
         <v>Add</v>
       </c>
+      <c r="Q193" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -10548,6 +10674,9 @@
       <c r="P194" t="str">
         <v>Add</v>
       </c>
+      <c r="Q194" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -10598,6 +10727,9 @@
       <c r="P195" t="str">
         <v>Add</v>
       </c>
+      <c r="Q195" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -10648,6 +10780,9 @@
       <c r="P196" t="str">
         <v>Add</v>
       </c>
+      <c r="Q196" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -10698,6 +10833,9 @@
       <c r="P197" t="str">
         <v>Add</v>
       </c>
+      <c r="Q197" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -10748,6 +10886,9 @@
       <c r="P198" t="str">
         <v>Add</v>
       </c>
+      <c r="Q198" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -10798,6 +10939,9 @@
       <c r="P199" t="str">
         <v>Add</v>
       </c>
+      <c r="Q199" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -10848,6 +10992,9 @@
       <c r="P200" t="str">
         <v>Add</v>
       </c>
+      <c r="Q200" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -10898,6 +11045,9 @@
       <c r="P201" t="str">
         <v>Add</v>
       </c>
+      <c r="Q201" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -10948,6 +11098,9 @@
       <c r="P202" t="str">
         <v>Add</v>
       </c>
+      <c r="Q202" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -10998,6 +11151,9 @@
       <c r="P203" t="str">
         <v>Add</v>
       </c>
+      <c r="Q203" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -11048,6 +11204,9 @@
       <c r="P204" t="str">
         <v>Add</v>
       </c>
+      <c r="Q204" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -11098,6 +11257,9 @@
       <c r="P205" t="str">
         <v>Add</v>
       </c>
+      <c r="Q205" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -11148,6 +11310,9 @@
       <c r="P206" t="str">
         <v>Add</v>
       </c>
+      <c r="Q206" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -11198,6 +11363,9 @@
       <c r="P207" t="str">
         <v>Add</v>
       </c>
+      <c r="Q207" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -11248,6 +11416,9 @@
       <c r="P208" t="str">
         <v>Add</v>
       </c>
+      <c r="Q208" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -11298,6 +11469,9 @@
       <c r="P209" t="str">
         <v>Add</v>
       </c>
+      <c r="Q209" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -11348,6 +11522,9 @@
       <c r="P210" t="str">
         <v>Add</v>
       </c>
+      <c r="Q210" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -11398,6 +11575,9 @@
       <c r="P211" t="str">
         <v>Add</v>
       </c>
+      <c r="Q211" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -11448,6 +11628,9 @@
       <c r="P212" t="str">
         <v>Add</v>
       </c>
+      <c r="Q212" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -11498,6 +11681,9 @@
       <c r="P213" t="str">
         <v>Add</v>
       </c>
+      <c r="Q213" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -11548,6 +11734,9 @@
       <c r="P214" t="str">
         <v>Add</v>
       </c>
+      <c r="Q214" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -11598,6 +11787,9 @@
       <c r="P215" t="str">
         <v>Add</v>
       </c>
+      <c r="Q215" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -11648,6 +11840,9 @@
       <c r="P216" t="str">
         <v>Add</v>
       </c>
+      <c r="Q216" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -11698,6 +11893,9 @@
       <c r="P217" t="str">
         <v>Add</v>
       </c>
+      <c r="Q217" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -11748,6 +11946,9 @@
       <c r="P218" t="str">
         <v>Add</v>
       </c>
+      <c r="Q218" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -11798,6 +11999,9 @@
       <c r="P219" t="str">
         <v>Add</v>
       </c>
+      <c r="Q219" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -11848,6 +12052,9 @@
       <c r="P220" t="str">
         <v>Add</v>
       </c>
+      <c r="Q220" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -11898,6 +12105,9 @@
       <c r="P221" t="str">
         <v>Add</v>
       </c>
+      <c r="Q221" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -11948,6 +12158,9 @@
       <c r="P222" t="str">
         <v>Add</v>
       </c>
+      <c r="Q222" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -11998,6 +12211,9 @@
       <c r="P223" t="str">
         <v>Add</v>
       </c>
+      <c r="Q223" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -12048,6 +12264,9 @@
       <c r="P224" t="str">
         <v>Add</v>
       </c>
+      <c r="Q224" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -12098,6 +12317,9 @@
       <c r="P225" t="str">
         <v>Add</v>
       </c>
+      <c r="Q225" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -12148,6 +12370,9 @@
       <c r="P226" t="str">
         <v>Add</v>
       </c>
+      <c r="Q226" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -12198,6 +12423,9 @@
       <c r="P227" t="str">
         <v>Add</v>
       </c>
+      <c r="Q227" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -12248,6 +12476,9 @@
       <c r="P228" t="str">
         <v>Add</v>
       </c>
+      <c r="Q228" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -12298,6 +12529,9 @@
       <c r="P229" t="str">
         <v>Add</v>
       </c>
+      <c r="Q229" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -12348,6 +12582,9 @@
       <c r="P230" t="str">
         <v>Add</v>
       </c>
+      <c r="Q230" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -12397,6 +12634,9 @@
       </c>
       <c r="P231" t="str">
         <v>Add</v>
+      </c>
+      <c r="Q231" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
feat: update row range in fetch-worker.js and correct numFound value in results_manual.json
</commit_message>
<xml_diff>
--- a/volume/output_manual.xlsx
+++ b/volume/output_manual.xlsx
@@ -25994,6 +25994,9 @@
       <c r="P483" t="str">
         <v>Add</v>
       </c>
+      <c r="Q483" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="str">
@@ -26044,6 +26047,9 @@
       <c r="P484" t="str">
         <v>Add</v>
       </c>
+      <c r="Q484" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="str">
@@ -26094,6 +26100,9 @@
       <c r="P485" t="str">
         <v>Add</v>
       </c>
+      <c r="Q485" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="486">
       <c r="A486" t="str">
@@ -26144,6 +26153,9 @@
       <c r="P486" t="str">
         <v>Add</v>
       </c>
+      <c r="Q486" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="str">
@@ -26194,6 +26206,9 @@
       <c r="P487" t="str">
         <v>Add</v>
       </c>
+      <c r="Q487" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="488">
       <c r="A488" t="str">
@@ -26244,6 +26259,9 @@
       <c r="P488" t="str">
         <v>Add</v>
       </c>
+      <c r="Q488" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="str">
@@ -26294,6 +26312,9 @@
       <c r="P489" t="str">
         <v>Add</v>
       </c>
+      <c r="Q489" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="str">
@@ -26344,6 +26365,9 @@
       <c r="P490" t="str">
         <v>Add</v>
       </c>
+      <c r="Q490" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="str">
@@ -26394,6 +26418,9 @@
       <c r="P491" t="str">
         <v>Add</v>
       </c>
+      <c r="Q491" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="str">
@@ -26444,6 +26471,9 @@
       <c r="P492" t="str">
         <v>Add</v>
       </c>
+      <c r="Q492" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="str">
@@ -26494,6 +26524,9 @@
       <c r="P493" t="str">
         <v>Add</v>
       </c>
+      <c r="Q493" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="str">
@@ -26544,6 +26577,9 @@
       <c r="P494" t="str">
         <v>Add</v>
       </c>
+      <c r="Q494" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="str">
@@ -26594,6 +26630,9 @@
       <c r="P495" t="str">
         <v>Add</v>
       </c>
+      <c r="Q495" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="496">
       <c r="A496" t="str">
@@ -26644,6 +26683,9 @@
       <c r="P496" t="str">
         <v>Add</v>
       </c>
+      <c r="Q496" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="str">
@@ -26694,6 +26736,9 @@
       <c r="P497" t="str">
         <v>Add</v>
       </c>
+      <c r="Q497" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="str">
@@ -26744,6 +26789,9 @@
       <c r="P498" t="str">
         <v>Add</v>
       </c>
+      <c r="Q498" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="str">
@@ -26794,6 +26842,9 @@
       <c r="P499" t="str">
         <v>Add</v>
       </c>
+      <c r="Q499" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="str">
@@ -26844,6 +26895,9 @@
       <c r="P500" t="str">
         <v>Add</v>
       </c>
+      <c r="Q500" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="str">
@@ -26894,6 +26948,9 @@
       <c r="P501" t="str">
         <v>Add</v>
       </c>
+      <c r="Q501" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="str">
@@ -26944,6 +27001,9 @@
       <c r="P502" t="str">
         <v>Add</v>
       </c>
+      <c r="Q502" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="503">
       <c r="A503" t="str">
@@ -26994,6 +27054,9 @@
       <c r="P503" t="str">
         <v>Add</v>
       </c>
+      <c r="Q503" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="504">
       <c r="A504" t="str">
@@ -27044,6 +27107,9 @@
       <c r="P504" t="str">
         <v>Add</v>
       </c>
+      <c r="Q504" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="505">
       <c r="A505" t="str">
@@ -27094,6 +27160,9 @@
       <c r="P505" t="str">
         <v>Add</v>
       </c>
+      <c r="Q505" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="506">
       <c r="A506" t="str">
@@ -27144,6 +27213,9 @@
       <c r="P506" t="str">
         <v>Add</v>
       </c>
+      <c r="Q506" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="507">
       <c r="A507" t="str">
@@ -27194,6 +27266,9 @@
       <c r="P507" t="str">
         <v>Add</v>
       </c>
+      <c r="Q507" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="508">
       <c r="A508" t="str">
@@ -27244,6 +27319,9 @@
       <c r="P508" t="str">
         <v>Add</v>
       </c>
+      <c r="Q508" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="509">
       <c r="A509" t="str">
@@ -27294,6 +27372,9 @@
       <c r="P509" t="str">
         <v>Add</v>
       </c>
+      <c r="Q509" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="str">
@@ -27344,6 +27425,9 @@
       <c r="P510" t="str">
         <v>Add</v>
       </c>
+      <c r="Q510" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="511">
       <c r="A511" t="str">
@@ -27394,6 +27478,9 @@
       <c r="P511" t="str">
         <v>Add</v>
       </c>
+      <c r="Q511" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="512">
       <c r="A512" t="str">
@@ -27444,6 +27531,9 @@
       <c r="P512" t="str">
         <v>Add</v>
       </c>
+      <c r="Q512" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="513">
       <c r="A513" t="str">
@@ -27494,6 +27584,9 @@
       <c r="P513" t="str">
         <v>Add</v>
       </c>
+      <c r="Q513" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="514">
       <c r="A514" t="str">
@@ -27544,6 +27637,9 @@
       <c r="P514" t="str">
         <v>Add</v>
       </c>
+      <c r="Q514" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="str">
@@ -27594,6 +27690,9 @@
       <c r="P515" t="str">
         <v>Add</v>
       </c>
+      <c r="Q515" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="516">
       <c r="A516" t="str">
@@ -27644,6 +27743,9 @@
       <c r="P516" t="str">
         <v>Add</v>
       </c>
+      <c r="Q516" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="517">
       <c r="A517" t="str">
@@ -27694,6 +27796,9 @@
       <c r="P517" t="str">
         <v>Add</v>
       </c>
+      <c r="Q517" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="518">
       <c r="A518" t="str">
@@ -27744,6 +27849,9 @@
       <c r="P518" t="str">
         <v>Add</v>
       </c>
+      <c r="Q518" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="519">
       <c r="A519" t="str">
@@ -27794,6 +27902,9 @@
       <c r="P519" t="str">
         <v>Add</v>
       </c>
+      <c r="Q519" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="520">
       <c r="A520" t="str">
@@ -27844,6 +27955,9 @@
       <c r="P520" t="str">
         <v>Add</v>
       </c>
+      <c r="Q520" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="521">
       <c r="A521" t="str">
@@ -27894,6 +28008,9 @@
       <c r="P521" t="str">
         <v>Add</v>
       </c>
+      <c r="Q521" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="522">
       <c r="A522" t="str">
@@ -27944,6 +28061,9 @@
       <c r="P522" t="str">
         <v>Add</v>
       </c>
+      <c r="Q522" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="523">
       <c r="A523" t="str">
@@ -27994,6 +28114,9 @@
       <c r="P523" t="str">
         <v>Add</v>
       </c>
+      <c r="Q523" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="524">
       <c r="A524" t="str">
@@ -28044,6 +28167,9 @@
       <c r="P524" t="str">
         <v>Add</v>
       </c>
+      <c r="Q524" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="525">
       <c r="A525" t="str">
@@ -28094,6 +28220,9 @@
       <c r="P525" t="str">
         <v>Add</v>
       </c>
+      <c r="Q525" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="526">
       <c r="A526" t="str">
@@ -28144,6 +28273,9 @@
       <c r="P526" t="str">
         <v>Add</v>
       </c>
+      <c r="Q526" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="527">
       <c r="A527" t="str">
@@ -28194,6 +28326,9 @@
       <c r="P527" t="str">
         <v>Add</v>
       </c>
+      <c r="Q527" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="528">
       <c r="A528" t="str">
@@ -28244,6 +28379,9 @@
       <c r="P528" t="str">
         <v>Add</v>
       </c>
+      <c r="Q528" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="529">
       <c r="A529" t="str">
@@ -28294,6 +28432,9 @@
       <c r="P529" t="str">
         <v>Add</v>
       </c>
+      <c r="Q529" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="530">
       <c r="A530" t="str">
@@ -28344,6 +28485,9 @@
       <c r="P530" t="str">
         <v>Add</v>
       </c>
+      <c r="Q530" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="531">
       <c r="A531" t="str">
@@ -28394,6 +28538,9 @@
       <c r="P531" t="str">
         <v>Add</v>
       </c>
+      <c r="Q531" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="532">
       <c r="A532" t="str">
@@ -28443,6 +28590,9 @@
       </c>
       <c r="P532" t="str">
         <v>Add</v>
+      </c>
+      <c r="Q532" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="533">

</xml_diff>

<commit_message>
feat: update fetch-worker.js with new bearer token and add stock entries to results_manual.json
</commit_message>
<xml_diff>
--- a/volume/output_manual.xlsx
+++ b/volume/output_manual.xlsx
@@ -28644,6 +28644,9 @@
       <c r="P533" t="str">
         <v>Add</v>
       </c>
+      <c r="Q533" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="534">
       <c r="A534" t="str">
@@ -28694,6 +28697,9 @@
       <c r="P534" t="str">
         <v>Add</v>
       </c>
+      <c r="Q534" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="str">
@@ -28744,6 +28750,9 @@
       <c r="P535" t="str">
         <v>Add</v>
       </c>
+      <c r="Q535" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="536">
       <c r="A536" t="str">
@@ -28794,6 +28803,9 @@
       <c r="P536" t="str">
         <v>Add</v>
       </c>
+      <c r="Q536" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="537">
       <c r="A537" t="str">
@@ -28844,6 +28856,9 @@
       <c r="P537" t="str">
         <v>Add</v>
       </c>
+      <c r="Q537" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="538">
       <c r="A538" t="str">
@@ -28894,6 +28909,9 @@
       <c r="P538" t="str">
         <v>Add</v>
       </c>
+      <c r="Q538" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="539">
       <c r="A539" t="str">
@@ -28944,6 +28962,9 @@
       <c r="P539" t="str">
         <v>Add</v>
       </c>
+      <c r="Q539" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="540">
       <c r="A540" t="str">
@@ -28994,6 +29015,9 @@
       <c r="P540" t="str">
         <v>Add</v>
       </c>
+      <c r="Q540" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="str">
@@ -29044,6 +29068,9 @@
       <c r="P541" t="str">
         <v>Add</v>
       </c>
+      <c r="Q541" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="str">
@@ -29094,6 +29121,9 @@
       <c r="P542" t="str">
         <v>Add</v>
       </c>
+      <c r="Q542" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="543">
       <c r="A543" t="str">
@@ -29144,6 +29174,9 @@
       <c r="P543" t="str">
         <v>Add</v>
       </c>
+      <c r="Q543" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="544">
       <c r="A544" t="str">
@@ -29194,6 +29227,9 @@
       <c r="P544" t="str">
         <v>Add</v>
       </c>
+      <c r="Q544" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="str">
@@ -29244,6 +29280,9 @@
       <c r="P545" t="str">
         <v>Add</v>
       </c>
+      <c r="Q545" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="546">
       <c r="A546" t="str">
@@ -29294,6 +29333,9 @@
       <c r="P546" t="str">
         <v>Add</v>
       </c>
+      <c r="Q546" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="547">
       <c r="A547" t="str">
@@ -29344,6 +29386,9 @@
       <c r="P547" t="str">
         <v>Add</v>
       </c>
+      <c r="Q547" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="548">
       <c r="A548" t="str">
@@ -29394,6 +29439,9 @@
       <c r="P548" t="str">
         <v>Add</v>
       </c>
+      <c r="Q548" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="549">
       <c r="A549" t="str">
@@ -29444,6 +29492,9 @@
       <c r="P549" t="str">
         <v>Add</v>
       </c>
+      <c r="Q549" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="550">
       <c r="A550" t="str">
@@ -29494,6 +29545,9 @@
       <c r="P550" t="str">
         <v>Add</v>
       </c>
+      <c r="Q550" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="551">
       <c r="A551" t="str">
@@ -29544,6 +29598,9 @@
       <c r="P551" t="str">
         <v>Add</v>
       </c>
+      <c r="Q551" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="552">
       <c r="A552" t="str">
@@ -29594,6 +29651,9 @@
       <c r="P552" t="str">
         <v>Add</v>
       </c>
+      <c r="Q552" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="553">
       <c r="A553" t="str">
@@ -29644,6 +29704,9 @@
       <c r="P553" t="str">
         <v>Add</v>
       </c>
+      <c r="Q553" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="554">
       <c r="A554" t="str">
@@ -29694,6 +29757,9 @@
       <c r="P554" t="str">
         <v>Add</v>
       </c>
+      <c r="Q554" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="555">
       <c r="A555" t="str">
@@ -29744,6 +29810,9 @@
       <c r="P555" t="str">
         <v>Add</v>
       </c>
+      <c r="Q555" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="556">
       <c r="A556" t="str">
@@ -29794,6 +29863,9 @@
       <c r="P556" t="str">
         <v>Add</v>
       </c>
+      <c r="Q556" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="557">
       <c r="A557" t="str">
@@ -29844,6 +29916,9 @@
       <c r="P557" t="str">
         <v>Add</v>
       </c>
+      <c r="Q557" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="558">
       <c r="A558" t="str">
@@ -29894,6 +29969,9 @@
       <c r="P558" t="str">
         <v>Add</v>
       </c>
+      <c r="Q558" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="559">
       <c r="A559" t="str">
@@ -29944,6 +30022,9 @@
       <c r="P559" t="str">
         <v>Add</v>
       </c>
+      <c r="Q559" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="560">
       <c r="A560" t="str">
@@ -29994,6 +30075,9 @@
       <c r="P560" t="str">
         <v>Add</v>
       </c>
+      <c r="Q560" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="561">
       <c r="A561" t="str">
@@ -30044,6 +30128,9 @@
       <c r="P561" t="str">
         <v>Add</v>
       </c>
+      <c r="Q561" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="562">
       <c r="A562" t="str">
@@ -30094,6 +30181,9 @@
       <c r="P562" t="str">
         <v>Add</v>
       </c>
+      <c r="Q562" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="563">
       <c r="A563" t="str">
@@ -30144,6 +30234,9 @@
       <c r="P563" t="str">
         <v>Add</v>
       </c>
+      <c r="Q563" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="564">
       <c r="A564" t="str">
@@ -30194,6 +30287,9 @@
       <c r="P564" t="str">
         <v>Add</v>
       </c>
+      <c r="Q564" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="565">
       <c r="A565" t="str">
@@ -30244,6 +30340,9 @@
       <c r="P565" t="str">
         <v>Add</v>
       </c>
+      <c r="Q565" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="566">
       <c r="A566" t="str">
@@ -30294,6 +30393,9 @@
       <c r="P566" t="str">
         <v>Add</v>
       </c>
+      <c r="Q566" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="567">
       <c r="A567" t="str">
@@ -30344,6 +30446,9 @@
       <c r="P567" t="str">
         <v>Add</v>
       </c>
+      <c r="Q567" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="568">
       <c r="A568" t="str">
@@ -30394,6 +30499,9 @@
       <c r="P568" t="str">
         <v>Add</v>
       </c>
+      <c r="Q568" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="569">
       <c r="A569" t="str">
@@ -30444,6 +30552,9 @@
       <c r="P569" t="str">
         <v>Add</v>
       </c>
+      <c r="Q569" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="570">
       <c r="A570" t="str">
@@ -30494,6 +30605,9 @@
       <c r="P570" t="str">
         <v>Add</v>
       </c>
+      <c r="Q570" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="571">
       <c r="A571" t="str">
@@ -30544,6 +30658,9 @@
       <c r="P571" t="str">
         <v>Add</v>
       </c>
+      <c r="Q571" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="572">
       <c r="A572" t="str">
@@ -30594,6 +30711,9 @@
       <c r="P572" t="str">
         <v>Add</v>
       </c>
+      <c r="Q572" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="573">
       <c r="A573" t="str">
@@ -30644,6 +30764,9 @@
       <c r="P573" t="str">
         <v>Add</v>
       </c>
+      <c r="Q573" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="str">
@@ -30694,6 +30817,9 @@
       <c r="P574" t="str">
         <v>Add</v>
       </c>
+      <c r="Q574" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="575">
       <c r="A575" t="str">
@@ -30744,6 +30870,9 @@
       <c r="P575" t="str">
         <v>Add</v>
       </c>
+      <c r="Q575" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="576">
       <c r="A576" t="str">
@@ -30794,6 +30923,9 @@
       <c r="P576" t="str">
         <v>Add</v>
       </c>
+      <c r="Q576" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="str">
@@ -30844,6 +30976,9 @@
       <c r="P577" t="str">
         <v>Add</v>
       </c>
+      <c r="Q577" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="str">
@@ -30894,6 +31029,9 @@
       <c r="P578" t="str">
         <v>Add</v>
       </c>
+      <c r="Q578" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="579">
       <c r="A579" t="str">
@@ -30944,6 +31082,9 @@
       <c r="P579" t="str">
         <v>Add</v>
       </c>
+      <c r="Q579" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="580">
       <c r="A580" t="str">
@@ -30994,6 +31135,9 @@
       <c r="P580" t="str">
         <v>Add</v>
       </c>
+      <c r="Q580" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="581">
       <c r="A581" t="str">
@@ -31044,6 +31188,9 @@
       <c r="P581" t="str">
         <v>Add</v>
       </c>
+      <c r="Q581" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="582">
       <c r="A582" t="str">
@@ -31093,6 +31240,9 @@
       </c>
       <c r="P582" t="str">
         <v>Add</v>
+      </c>
+      <c r="Q582" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="583">

</xml_diff>